<commit_message>
critical update to instructions
</commit_message>
<xml_diff>
--- a/STELLA-1.2/lab_spec_documents/Lab Spec Build Instructions.xlsx
+++ b/STELLA-1.2/lab_spec_documents/Lab Spec Build Instructions.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="267">
   <si>
     <t>STELLA Lab Spec parts</t>
   </si>
@@ -76,7 +76,7 @@
     <t>$ line</t>
   </si>
   <si>
-    <t>.STL</t>
+    <t>.STL details, or link to part</t>
   </si>
   <si>
     <t>C2</t>
@@ -166,9 +166,26 @@
     <t>Proto-Advantage LED2 - DIP adapter</t>
   </si>
   <si>
+    <t>Proto-Advantage</t>
+  </si>
+  <si>
     <t>Proto-Advantage small proto board</t>
   </si>
   <si>
+    <t>SBB1002-1</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://www.proto-advantage.com/store/product_info.php?products_id=200009</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">Socket header 3x1 pos </t>
   </si>
   <si>
@@ -184,10 +201,16 @@
     <t>Sparkfun mini proto board</t>
   </si>
   <si>
-    <t>Stacking header 6 pos</t>
-  </si>
-  <si>
-    <t>Stacking headers, 6 pos</t>
+    <t>Socket header 6 pos</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>need to find socket headers of correct height</t>
+  </si>
+  <si>
+    <t>Socket headers, 6 pos</t>
   </si>
   <si>
     <t>White LED panel</t>
@@ -298,9 +321,6 @@
     <t>LS-C2 Cuvette optics</t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
     <t>LS-C2 Assembly drawing</t>
   </si>
   <si>
@@ -340,6 +360,9 @@
     <t xml:space="preserve">What color? </t>
   </si>
   <si>
+    <t>Note</t>
+  </si>
+  <si>
     <t>Get board</t>
   </si>
   <si>
@@ -367,12 +390,15 @@
     <t>Install transistors</t>
   </si>
   <si>
-    <t>2N2222 or PN2222</t>
+    <t>2N2222 or PN2222ABU</t>
   </si>
   <si>
     <t>All flats towards J: B12-13-14; B16-17-18; G12-13-14; G16-17-18</t>
   </si>
   <si>
+    <t>Solder the center pin first, then straighten the body before soldering the other two pins</t>
+  </si>
+  <si>
     <t>Install shunt resistors</t>
   </si>
   <si>
@@ -400,7 +426,10 @@
     <t>C11-E13, C15-E17; H11-J13; H15-J17</t>
   </si>
   <si>
-    <t>Install stacking headers for devices</t>
+    <t xml:space="preserve">49.9Ω in photos. Either value is OK. </t>
+  </si>
+  <si>
+    <t>Install socket headers for devices</t>
   </si>
   <si>
     <t>6 pos, 4 places</t>
@@ -415,13 +444,13 @@
     <t>3x3, 2 places</t>
   </si>
   <si>
-    <t>ON BACK: A, B, C x 1, 2, 3; H, i, J x 1, 2, 3</t>
+    <t>ON BACK: A,B,C x 1,2,3; H,i,J x 1,2,3</t>
   </si>
   <si>
     <t>3 pos, 3 places</t>
   </si>
   <si>
-    <t>ON BACK: SCL 1, 2, 3; GND 1, 2, 3; 3V 1, 2, 3</t>
+    <t>ON BACK: SDA 1,2,3; GND 1,2,3; 3V 1,2,3</t>
   </si>
   <si>
     <t>Install ground wires</t>
@@ -830,7 +859,7 @@
   <numFmts count="1">
     <numFmt numFmtId="0" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -843,6 +872,12 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Helvetica Neue"/>
+    </font>
+    <font>
+      <u val="single"/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
@@ -1174,6 +1209,21 @@
         <color indexed="10"/>
       </left>
       <right style="thin">
+        <color indexed="10"/>
+      </right>
+      <top style="thin">
+        <color indexed="10"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="17"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right style="thin">
         <color indexed="17"/>
       </right>
       <top style="medium">
@@ -1289,28 +1339,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="17"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1395,12 +1430,15 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1410,6 +1448,9 @@
     <xf numFmtId="0" fontId="0" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1422,25 +1463,37 @@
     <xf numFmtId="0" fontId="0" borderId="16" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="17" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" borderId="17" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="18" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="18" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" borderId="19" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="19" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" borderId="19" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="20" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="20" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" borderId="21" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="9" borderId="19" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" borderId="21" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="20" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="10" borderId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="10" borderId="22" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="22" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" borderId="23" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" borderId="23" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="11" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -1458,16 +1511,16 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="23" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="24" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="24" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="25" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="25" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" borderId="17" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
@@ -1482,7 +1535,7 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="10" borderId="19" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="10" borderId="20" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
@@ -3443,7 +3496,9 @@
       <c r="F32" t="s" s="11">
         <v>22</v>
       </c>
-      <c r="G32" s="13"/>
+      <c r="G32" t="s" s="11">
+        <v>41</v>
+      </c>
       <c r="H32" s="13"/>
       <c r="I32" s="13"/>
       <c r="J32" s="12" cm="1">
@@ -3471,7 +3526,9 @@
       <c r="F33" t="s" s="11">
         <v>22</v>
       </c>
-      <c r="G33" s="13"/>
+      <c r="G33" t="s" s="11">
+        <v>41</v>
+      </c>
       <c r="H33" s="13"/>
       <c r="I33" s="13"/>
       <c r="J33" s="12" cm="1">
@@ -3488,7 +3545,7 @@
         <v>12</v>
       </c>
       <c r="C34" t="s" s="11">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D34" s="12">
         <v>1</v>
@@ -3499,14 +3556,22 @@
       <c r="F34" t="s" s="11">
         <v>22</v>
       </c>
-      <c r="G34" s="13"/>
-      <c r="H34" s="13"/>
-      <c r="I34" s="13"/>
+      <c r="G34" t="s" s="11">
+        <v>41</v>
+      </c>
+      <c r="H34" t="s" s="11">
+        <v>43</v>
+      </c>
+      <c r="I34" s="12">
+        <v>1</v>
+      </c>
       <c r="J34" s="12" cm="1">
         <f t="array" ref="J34">I34*D34</f>
-        <v>0</v>
-      </c>
-      <c r="K34" s="13"/>
+        <v>1</v>
+      </c>
+      <c r="K34" t="s" s="11">
+        <v>44</v>
+      </c>
     </row>
     <row r="35" ht="20.05" customHeight="1">
       <c r="A35" s="9">
@@ -3516,7 +3581,7 @@
         <v>16</v>
       </c>
       <c r="C35" t="s" s="11">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D35" s="12">
         <v>1</v>
@@ -3527,14 +3592,22 @@
       <c r="F35" t="s" s="11">
         <v>22</v>
       </c>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="13"/>
+      <c r="G35" t="s" s="11">
+        <v>41</v>
+      </c>
+      <c r="H35" t="s" s="11">
+        <v>43</v>
+      </c>
+      <c r="I35" s="12">
+        <v>1</v>
+      </c>
       <c r="J35" s="12" cm="1">
         <f t="array" ref="J35">I35*D35</f>
-        <v>0</v>
-      </c>
-      <c r="K35" s="13"/>
+        <v>1</v>
+      </c>
+      <c r="K35" t="s" s="11">
+        <v>44</v>
+      </c>
     </row>
     <row r="36" ht="20.05" customHeight="1">
       <c r="A36" s="9">
@@ -3544,7 +3617,7 @@
         <v>19</v>
       </c>
       <c r="C36" t="s" s="11">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D36" s="12">
         <v>1</v>
@@ -3572,7 +3645,7 @@
         <v>19</v>
       </c>
       <c r="C37" t="s" s="11">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D37" s="12">
         <v>1</v>
@@ -3600,7 +3673,7 @@
         <v>19</v>
       </c>
       <c r="C38" t="s" s="11">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D38" s="12">
         <v>2</v>
@@ -3628,7 +3701,7 @@
         <v>16</v>
       </c>
       <c r="C39" t="s" s="11">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D39" s="12">
         <v>1</v>
@@ -3656,7 +3729,7 @@
         <v>12</v>
       </c>
       <c r="C40" t="s" s="11">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D40" s="12">
         <v>2</v>
@@ -3684,7 +3757,7 @@
         <v>16</v>
       </c>
       <c r="C41" t="s" s="11">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D41" s="12">
         <v>1</v>
@@ -3712,7 +3785,7 @@
         <v>12</v>
       </c>
       <c r="C42" t="s" s="11">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D42" s="12">
         <v>1</v>
@@ -3724,13 +3797,17 @@
         <v>22</v>
       </c>
       <c r="G42" s="13"/>
-      <c r="H42" s="13"/>
+      <c r="H42" t="s" s="11">
+        <v>51</v>
+      </c>
       <c r="I42" s="13"/>
       <c r="J42" s="12" cm="1">
         <f t="array" ref="J42">I42*D42</f>
         <v>0</v>
       </c>
-      <c r="K42" s="13"/>
+      <c r="K42" t="s" s="11">
+        <v>52</v>
+      </c>
     </row>
     <row r="43" ht="20.05" customHeight="1">
       <c r="A43" s="9">
@@ -3740,7 +3817,7 @@
         <v>19</v>
       </c>
       <c r="C43" t="s" s="11">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="D43" s="12">
         <v>4</v>
@@ -3752,13 +3829,17 @@
         <v>22</v>
       </c>
       <c r="G43" s="13"/>
-      <c r="H43" s="13"/>
+      <c r="H43" t="s" s="11">
+        <v>51</v>
+      </c>
       <c r="I43" s="13"/>
       <c r="J43" s="12" cm="1">
         <f t="array" ref="J43">I43*D43</f>
         <v>0</v>
       </c>
-      <c r="K43" s="13"/>
+      <c r="K43" t="s" s="11">
+        <v>52</v>
+      </c>
     </row>
     <row r="44" ht="20.05" customHeight="1">
       <c r="A44" s="9">
@@ -3768,7 +3849,7 @@
         <v>12</v>
       </c>
       <c r="C44" t="s" s="11">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D44" s="12">
         <v>1</v>
@@ -3796,7 +3877,7 @@
         <v>19</v>
       </c>
       <c r="C45" t="s" s="11">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D45" s="12">
         <v>1</v>
@@ -3805,7 +3886,7 @@
         <v>21</v>
       </c>
       <c r="F45" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G45" s="13"/>
       <c r="H45" s="13"/>
@@ -3815,7 +3896,7 @@
         <v>0</v>
       </c>
       <c r="K45" t="s" s="11">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="46" ht="20.05" customHeight="1">
@@ -3826,7 +3907,7 @@
         <v>12</v>
       </c>
       <c r="C46" t="s" s="11">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D46" s="12">
         <v>1</v>
@@ -3835,7 +3916,7 @@
         <v>14</v>
       </c>
       <c r="F46" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G46" s="13"/>
       <c r="H46" s="13"/>
@@ -3845,7 +3926,7 @@
         <v>0</v>
       </c>
       <c r="K46" t="s" s="11">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="47" ht="20.05" customHeight="1">
@@ -3856,7 +3937,7 @@
         <v>12</v>
       </c>
       <c r="C47" t="s" s="11">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D47" s="12">
         <v>1</v>
@@ -3865,7 +3946,7 @@
         <v>14</v>
       </c>
       <c r="F47" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G47" s="13"/>
       <c r="H47" s="13"/>
@@ -3875,7 +3956,7 @@
         <v>0</v>
       </c>
       <c r="K47" t="s" s="11">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="48" ht="20.05" customHeight="1">
@@ -3886,7 +3967,7 @@
         <v>12</v>
       </c>
       <c r="C48" t="s" s="11">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D48" s="12">
         <v>1</v>
@@ -3895,7 +3976,7 @@
         <v>14</v>
       </c>
       <c r="F48" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G48" s="13"/>
       <c r="H48" s="13"/>
@@ -3905,7 +3986,7 @@
         <v>0</v>
       </c>
       <c r="K48" t="s" s="11">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="49" ht="20.05" customHeight="1">
@@ -3916,7 +3997,7 @@
         <v>12</v>
       </c>
       <c r="C49" t="s" s="11">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D49" s="12">
         <v>1</v>
@@ -3925,7 +4006,7 @@
         <v>14</v>
       </c>
       <c r="F49" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G49" s="13"/>
       <c r="H49" s="13"/>
@@ -3935,7 +4016,7 @@
         <v>0</v>
       </c>
       <c r="K49" t="s" s="11">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="50" ht="20.05" customHeight="1">
@@ -3946,7 +4027,7 @@
         <v>12</v>
       </c>
       <c r="C50" t="s" s="11">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D50" s="12">
         <v>1</v>
@@ -3955,7 +4036,7 @@
         <v>14</v>
       </c>
       <c r="F50" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G50" s="13"/>
       <c r="H50" s="13"/>
@@ -3965,7 +4046,7 @@
         <v>0</v>
       </c>
       <c r="K50" t="s" s="11">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="51" ht="20.05" customHeight="1">
@@ -3976,7 +4057,7 @@
         <v>12</v>
       </c>
       <c r="C51" t="s" s="11">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D51" s="12">
         <v>1</v>
@@ -3985,7 +4066,7 @@
         <v>14</v>
       </c>
       <c r="F51" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G51" s="13"/>
       <c r="H51" s="13"/>
@@ -3995,7 +4076,7 @@
         <v>0</v>
       </c>
       <c r="K51" t="s" s="11">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="52" ht="20.05" customHeight="1">
@@ -4006,7 +4087,7 @@
         <v>12</v>
       </c>
       <c r="C52" t="s" s="11">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D52" s="12">
         <v>1</v>
@@ -4015,7 +4096,7 @@
         <v>14</v>
       </c>
       <c r="F52" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G52" s="13"/>
       <c r="H52" s="13"/>
@@ -4025,7 +4106,7 @@
         <v>0</v>
       </c>
       <c r="K52" t="s" s="11">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="53" ht="20.05" customHeight="1">
@@ -4036,7 +4117,7 @@
         <v>12</v>
       </c>
       <c r="C53" t="s" s="11">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D53" s="12">
         <v>1</v>
@@ -4045,7 +4126,7 @@
         <v>14</v>
       </c>
       <c r="F53" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G53" s="13"/>
       <c r="H53" s="13"/>
@@ -4055,7 +4136,7 @@
         <v>0</v>
       </c>
       <c r="K53" t="s" s="11">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="54" ht="20.05" customHeight="1">
@@ -4066,7 +4147,7 @@
         <v>12</v>
       </c>
       <c r="C54" t="s" s="11">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D54" s="12">
         <v>1</v>
@@ -4075,7 +4156,7 @@
         <v>14</v>
       </c>
       <c r="F54" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G54" s="13"/>
       <c r="H54" s="13"/>
@@ -4085,7 +4166,7 @@
         <v>0</v>
       </c>
       <c r="K54" t="s" s="11">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="55" ht="20.05" customHeight="1">
@@ -4096,7 +4177,7 @@
         <v>12</v>
       </c>
       <c r="C55" t="s" s="11">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D55" s="12">
         <v>1</v>
@@ -4105,7 +4186,7 @@
         <v>14</v>
       </c>
       <c r="F55" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G55" s="13"/>
       <c r="H55" s="13"/>
@@ -4115,7 +4196,7 @@
         <v>0</v>
       </c>
       <c r="K55" t="s" s="11">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="56" ht="20.05" customHeight="1">
@@ -4126,7 +4207,7 @@
         <v>16</v>
       </c>
       <c r="C56" t="s" s="11">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D56" s="12">
         <v>1</v>
@@ -4135,7 +4216,7 @@
         <v>18</v>
       </c>
       <c r="F56" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G56" s="13"/>
       <c r="H56" s="13"/>
@@ -4145,7 +4226,7 @@
         <v>0</v>
       </c>
       <c r="K56" t="s" s="11">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="57" ht="20.05" customHeight="1">
@@ -4156,7 +4237,7 @@
         <v>16</v>
       </c>
       <c r="C57" t="s" s="11">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D57" s="12">
         <v>1</v>
@@ -4165,7 +4246,7 @@
         <v>18</v>
       </c>
       <c r="F57" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G57" s="13"/>
       <c r="H57" s="13"/>
@@ -4175,7 +4256,7 @@
         <v>0</v>
       </c>
       <c r="K57" t="s" s="11">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="58" ht="20.05" customHeight="1">
@@ -4186,7 +4267,7 @@
         <v>16</v>
       </c>
       <c r="C58" t="s" s="11">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D58" s="12">
         <v>1</v>
@@ -4195,7 +4276,7 @@
         <v>18</v>
       </c>
       <c r="F58" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G58" s="13"/>
       <c r="H58" s="13"/>
@@ -4205,7 +4286,7 @@
         <v>0</v>
       </c>
       <c r="K58" t="s" s="11">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="59" ht="20.05" customHeight="1">
@@ -4216,7 +4297,7 @@
         <v>16</v>
       </c>
       <c r="C59" t="s" s="11">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D59" s="12">
         <v>1</v>
@@ -4225,7 +4306,7 @@
         <v>18</v>
       </c>
       <c r="F59" t="s" s="11">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G59" s="13"/>
       <c r="H59" s="13"/>
@@ -4235,7 +4316,7 @@
         <v>0</v>
       </c>
       <c r="K59" t="s" s="11">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="60" ht="20.25" customHeight="1">
@@ -4246,7 +4327,7 @@
         <v>16</v>
       </c>
       <c r="C60" t="s" s="16">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D60" s="17">
         <v>1</v>
@@ -4255,7 +4336,7 @@
         <v>18</v>
       </c>
       <c r="F60" t="s" s="16">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G60" s="18"/>
       <c r="H60" s="18"/>
@@ -4265,14 +4346,14 @@
         <v>0</v>
       </c>
       <c r="K60" t="s" s="16">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="61" ht="20.25" customHeight="1">
       <c r="A61" s="19"/>
       <c r="B61" s="19"/>
       <c r="C61" t="s" s="20">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D61" s="19"/>
       <c r="E61" s="19"/>
@@ -4282,7 +4363,7 @@
       <c r="I61" s="19"/>
       <c r="J61" s="21" cm="1">
         <f t="array" ref="J61">SUM(J3:J60)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K61" s="19"/>
     </row>
@@ -4290,6 +4371,10 @@
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="K34" r:id="rId1" location="" tooltip="" display="https://www.proto-advantage.com/store/product_info.php?products_id=200009"/>
+    <hyperlink ref="K35" r:id="rId2" location="" tooltip="" display="https://www.proto-advantage.com/store/product_info.php?products_id=200009"/>
+  </hyperlinks>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
   <headerFooter>
@@ -4315,16 +4400,16 @@
   <sheetData>
     <row r="1" ht="20.25" customHeight="1">
       <c r="A1" t="s" s="3">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B1" t="s" s="3">
         <v>2</v>
       </c>
       <c r="C1" t="s" s="3">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D1" t="s" s="3">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" ht="20.25" customHeight="1">
@@ -4335,10 +4420,10 @@
         <v>19</v>
       </c>
       <c r="C2" t="s" s="6">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D2" t="s" s="6">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" ht="20.05" customHeight="1">
@@ -4346,13 +4431,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s" s="10">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C3" t="s" s="11">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D3" t="s" s="11">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" ht="20.05" customHeight="1">
@@ -4360,13 +4445,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s" s="10">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C4" t="s" s="11">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D4" t="s" s="11">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" ht="20.05" customHeight="1">
@@ -4374,13 +4459,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s" s="10">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C5" t="s" s="11">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D5" t="s" s="11">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" ht="20.05" customHeight="1">
@@ -4388,13 +4473,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s" s="10">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C6" t="s" s="11">
+        <v>86</v>
+      </c>
+      <c r="D6" t="s" s="11">
         <v>81</v>
-      </c>
-      <c r="D6" t="s" s="11">
-        <v>76</v>
       </c>
     </row>
     <row r="7" ht="20.05" customHeight="1">
@@ -4402,13 +4487,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s" s="10">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C7" t="s" s="11">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D7" t="s" s="11">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" ht="20.05" customHeight="1">
@@ -4416,13 +4501,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s" s="10">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C8" t="s" s="11">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D8" t="s" s="11">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" ht="20.05" customHeight="1">
@@ -4430,13 +4515,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="s" s="10">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C9" t="s" s="11">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="D9" t="s" s="11">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" ht="20.05" customHeight="1">
@@ -4444,13 +4529,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="s" s="10">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C10" t="s" s="11">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="D10" t="s" s="11">
-        <v>85</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" ht="20.05" customHeight="1">
@@ -4458,13 +4543,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s" s="10">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C11" t="s" s="11">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D11" t="s" s="11">
-        <v>85</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" ht="20.05" customHeight="1">
@@ -4472,13 +4557,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="s" s="10">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C12" t="s" s="11">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D12" t="s" s="11">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" ht="20.05" customHeight="1">
@@ -4486,13 +4571,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s" s="10">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C13" t="s" s="11">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D13" t="s" s="11">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" ht="20.05" customHeight="1">
@@ -4500,13 +4585,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s" s="10">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C14" t="s" s="11">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D14" t="s" s="11">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" ht="20.05" customHeight="1">
@@ -4514,13 +4599,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="s" s="10">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C15" t="s" s="11">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D15" t="s" s="11">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" ht="20.05" customHeight="1">
@@ -4528,13 +4613,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s" s="10">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C16" t="s" s="11">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D16" t="s" s="11">
-        <v>85</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -4548,7 +4633,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:F25"/>
+  <dimension ref="A2:G25"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="8.10156" style="23" customWidth="1"/>
@@ -4557,105 +4642,116 @@
     <col min="4" max="4" width="61.1719" style="23" customWidth="1"/>
     <col min="5" max="5" width="16.3516" style="23" customWidth="1"/>
     <col min="6" max="6" width="11.7812" style="23" customWidth="1"/>
-    <col min="7" max="16384" width="16.3516" style="23" customWidth="1"/>
+    <col min="7" max="7" width="38.4531" style="23" customWidth="1"/>
+    <col min="8" max="16384" width="16.3516" style="23" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.65" customHeight="1">
       <c r="A1" t="s" s="2">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
     </row>
     <row r="2" ht="20.25" customHeight="1">
       <c r="A2" t="s" s="24">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B2" t="s" s="3">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s" s="3">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s" s="3">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E2" t="s" s="3">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F2" s="25"/>
+      <c r="G2" t="s" s="3">
+        <v>103</v>
+      </c>
     </row>
     <row r="3" ht="20.25" customHeight="1">
       <c r="A3" s="26">
         <v>1</v>
       </c>
       <c r="B3" t="s" s="5">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C3" t="s" s="6">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" t="s" s="6">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="F3" t="b" s="7">
         <v>0</v>
       </c>
+      <c r="G3" s="6"/>
     </row>
     <row r="4" ht="20.05" customHeight="1">
       <c r="A4" s="27">
         <v>2</v>
       </c>
       <c r="B4" t="s" s="10">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" t="s" s="11">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="E4" s="13"/>
       <c r="F4" t="b" s="12">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G4" s="11"/>
     </row>
     <row r="5" ht="20.05" customHeight="1">
       <c r="A5" s="27">
         <v>3</v>
       </c>
       <c r="B5" t="s" s="10">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C5" t="s" s="11">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="D5" t="s" s="11">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E5" s="13"/>
       <c r="F5" t="b" s="12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" ht="20.05" customHeight="1">
+        <v>1</v>
+      </c>
+      <c r="G5" s="11"/>
+    </row>
+    <row r="6" ht="32.05" customHeight="1">
       <c r="A6" s="27">
         <v>4</v>
       </c>
       <c r="B6" t="s" s="10">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C6" t="s" s="11">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D6" t="s" s="11">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="E6" s="13"/>
       <c r="F6" t="b" s="12">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="G6" t="s" s="11">
+        <v>115</v>
       </c>
     </row>
     <row r="7" ht="20.05" customHeight="1">
@@ -4663,53 +4759,58 @@
         <v>5</v>
       </c>
       <c r="B7" t="s" s="10">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="C7" t="s" s="11">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="D7" t="s" s="11">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="E7" s="13"/>
       <c r="F7" t="b" s="12">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G7" s="11"/>
     </row>
     <row r="8" ht="20.05" customHeight="1">
       <c r="A8" s="27">
         <v>6</v>
       </c>
       <c r="B8" t="s" s="10">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C8" t="s" s="11">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="D8" t="s" s="11">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="E8" s="13"/>
       <c r="F8" t="b" s="12">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G8" s="11"/>
     </row>
     <row r="9" ht="20.05" customHeight="1">
       <c r="A9" s="27">
         <v>7</v>
       </c>
       <c r="B9" t="s" s="10">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="C9" t="s" s="11">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="D9" t="s" s="11">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="E9" s="13"/>
       <c r="F9" t="b" s="12">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="G9" t="s" s="11">
+        <v>125</v>
       </c>
     </row>
     <row r="10" ht="20.05" customHeight="1">
@@ -4717,223 +4818,235 @@
         <v>8</v>
       </c>
       <c r="B10" t="s" s="10">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C10" t="s" s="11">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="D10" t="s" s="11">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="E10" s="13"/>
       <c r="F10" t="b" s="12">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G10" s="11"/>
     </row>
     <row r="11" ht="20.05" customHeight="1">
       <c r="A11" s="27">
         <v>9</v>
       </c>
       <c r="B11" t="s" s="10">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="C11" t="s" s="11">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="D11" t="s" s="11">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="E11" s="13"/>
       <c r="F11" t="b" s="12">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G11" s="11"/>
     </row>
     <row r="12" ht="20.05" customHeight="1">
       <c r="A12" s="27">
         <v>10</v>
       </c>
       <c r="B12" t="s" s="10">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="C12" t="s" s="11">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="D12" t="s" s="11">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="E12" s="13"/>
       <c r="F12" t="b" s="12">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G12" s="11"/>
     </row>
     <row r="13" ht="20.05" customHeight="1">
       <c r="A13" s="27">
         <v>11</v>
       </c>
       <c r="B13" t="s" s="10">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" t="s" s="11">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="E13" t="s" s="28">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="F13" t="b" s="29">
         <v>0</v>
       </c>
+      <c r="G13" s="30"/>
     </row>
     <row r="14" ht="20.05" customHeight="1">
       <c r="A14" s="27">
         <v>12</v>
       </c>
       <c r="B14" t="s" s="10">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="C14" s="13"/>
-      <c r="D14" t="s" s="30">
-        <v>131</v>
-      </c>
-      <c r="E14" t="s" s="31">
-        <v>132</v>
-      </c>
-      <c r="F14" t="b" s="32">
-        <v>0</v>
-      </c>
+      <c r="D14" t="s" s="31">
+        <v>138</v>
+      </c>
+      <c r="E14" t="s" s="32">
+        <v>139</v>
+      </c>
+      <c r="F14" t="b" s="33">
+        <v>0</v>
+      </c>
+      <c r="G14" s="34"/>
     </row>
     <row r="15" ht="20.85" customHeight="1">
       <c r="A15" s="27">
         <v>13</v>
       </c>
       <c r="B15" t="s" s="10">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" t="s" s="11">
-        <v>134</v>
-      </c>
-      <c r="E15" t="s" s="33">
-        <v>135</v>
+        <v>141</v>
+      </c>
+      <c r="E15" t="s" s="35">
+        <v>142</v>
       </c>
       <c r="F15" t="b" s="12">
         <v>0</v>
       </c>
+      <c r="G15" s="11"/>
     </row>
     <row r="16" ht="21.7" customHeight="1">
       <c r="A16" s="27">
         <v>14</v>
       </c>
       <c r="B16" t="s" s="10">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C16" s="13"/>
-      <c r="D16" t="s" s="34">
-        <v>137</v>
-      </c>
-      <c r="E16" t="s" s="35">
-        <v>138</v>
-      </c>
-      <c r="F16" t="b" s="36">
-        <v>0</v>
-      </c>
+      <c r="D16" t="s" s="36">
+        <v>144</v>
+      </c>
+      <c r="E16" t="s" s="37">
+        <v>145</v>
+      </c>
+      <c r="F16" t="b" s="38">
+        <v>0</v>
+      </c>
+      <c r="G16" s="39"/>
     </row>
     <row r="17" ht="20.85" customHeight="1">
       <c r="A17" s="27">
         <v>15</v>
       </c>
       <c r="B17" t="s" s="10">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="C17" s="13"/>
       <c r="D17" t="s" s="11">
-        <v>140</v>
-      </c>
-      <c r="E17" t="s" s="37">
-        <v>141</v>
-      </c>
-      <c r="F17" t="b" s="38">
-        <v>0</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="E17" t="s" s="40">
+        <v>148</v>
+      </c>
+      <c r="F17" t="b" s="41">
+        <v>0</v>
+      </c>
+      <c r="G17" s="42"/>
     </row>
     <row r="18" ht="20.05" customHeight="1">
       <c r="A18" s="27">
         <v>16</v>
       </c>
       <c r="B18" t="s" s="10">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C18" s="13"/>
       <c r="D18" t="s" s="11">
-        <v>143</v>
-      </c>
-      <c r="E18" t="s" s="39">
-        <v>144</v>
-      </c>
-      <c r="F18" t="b" s="40">
-        <v>0</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="E18" t="s" s="43">
+        <v>151</v>
+      </c>
+      <c r="F18" t="b" s="44">
+        <v>0</v>
+      </c>
+      <c r="G18" s="45"/>
     </row>
     <row r="19" ht="20.05" customHeight="1">
       <c r="A19" s="27">
         <v>17</v>
       </c>
       <c r="B19" t="s" s="10">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="C19" s="13"/>
       <c r="D19" t="s" s="11">
-        <v>146</v>
-      </c>
-      <c r="E19" t="s" s="41">
-        <v>147</v>
-      </c>
-      <c r="F19" t="b" s="40">
-        <v>0</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="E19" t="s" s="46">
+        <v>154</v>
+      </c>
+      <c r="F19" t="b" s="44">
+        <v>0</v>
+      </c>
+      <c r="G19" s="45"/>
     </row>
     <row r="20" ht="20.05" customHeight="1">
       <c r="A20" s="27">
         <v>18</v>
       </c>
       <c r="B20" t="s" s="10">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" t="s" s="11">
-        <v>149</v>
-      </c>
-      <c r="E20" t="s" s="42">
-        <v>150</v>
-      </c>
-      <c r="F20" t="b" s="43">
-        <v>0</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="E20" t="s" s="47">
+        <v>157</v>
+      </c>
+      <c r="F20" t="b" s="48">
+        <v>0</v>
+      </c>
+      <c r="G20" s="49"/>
     </row>
     <row r="21" ht="20.05" customHeight="1">
       <c r="A21" s="27">
         <v>19</v>
       </c>
       <c r="B21" t="s" s="10">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="C21" s="13"/>
-      <c r="D21" t="s" s="30">
-        <v>152</v>
-      </c>
-      <c r="E21" t="s" s="44">
-        <v>153</v>
-      </c>
-      <c r="F21" t="b" s="32">
-        <v>0</v>
-      </c>
+      <c r="D21" t="s" s="31">
+        <v>159</v>
+      </c>
+      <c r="E21" t="s" s="50">
+        <v>160</v>
+      </c>
+      <c r="F21" t="b" s="33">
+        <v>0</v>
+      </c>
+      <c r="G21" s="34"/>
     </row>
     <row r="22" ht="20.05" customHeight="1">
       <c r="A22" s="27">
         <v>20</v>
       </c>
       <c r="B22" t="s" s="10">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
@@ -4941,50 +5054,54 @@
       <c r="F22" t="b" s="12">
         <v>0</v>
       </c>
+      <c r="G22" s="11"/>
     </row>
     <row r="23" ht="20.05" customHeight="1">
       <c r="A23" s="27">
         <v>21</v>
       </c>
       <c r="B23" t="s" s="10">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" t="s" s="11">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E23" s="13"/>
       <c r="F23" t="b" s="12">
         <v>0</v>
       </c>
+      <c r="G23" s="11"/>
     </row>
     <row r="24" ht="20.05" customHeight="1">
       <c r="A24" s="27">
         <v>22</v>
       </c>
       <c r="B24" t="s" s="10">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C24" s="13"/>
       <c r="D24" t="s" s="11">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="E24" s="13"/>
       <c r="F24" t="b" s="12">
         <v>0</v>
       </c>
+      <c r="G24" s="11"/>
     </row>
     <row r="25" ht="20.05" customHeight="1">
-      <c r="A25" s="45"/>
-      <c r="B25" s="46"/>
+      <c r="A25" s="51"/>
+      <c r="B25" s="52"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
       <c r="E25" s="13"/>
       <c r="F25" s="13"/>
+      <c r="G25" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.277778" footer="0.277778"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="72" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
@@ -5002,17 +5119,17 @@
   <dimension ref="A2:E20"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="8.10156" style="47" customWidth="1"/>
-    <col min="2" max="2" width="43.5" style="47" customWidth="1"/>
-    <col min="3" max="3" width="34.2656" style="47" customWidth="1"/>
-    <col min="4" max="4" width="34.5" style="47" customWidth="1"/>
-    <col min="5" max="5" width="16.3516" style="47" customWidth="1"/>
-    <col min="6" max="16384" width="16.3516" style="47" customWidth="1"/>
+    <col min="1" max="1" width="8.10156" style="53" customWidth="1"/>
+    <col min="2" max="2" width="43.5" style="53" customWidth="1"/>
+    <col min="3" max="3" width="34.2656" style="53" customWidth="1"/>
+    <col min="4" max="4" width="34.5" style="53" customWidth="1"/>
+    <col min="5" max="5" width="16.3516" style="53" customWidth="1"/>
+    <col min="6" max="16384" width="16.3516" style="53" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.65" customHeight="1">
       <c r="A1" t="s" s="2">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5021,19 +5138,19 @@
     </row>
     <row r="2" ht="20.25" customHeight="1">
       <c r="A2" t="s" s="24">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B2" t="s" s="3">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s" s="3">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s" s="3">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E2" t="s" s="3">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" ht="20.25" customHeight="1">
@@ -5041,14 +5158,14 @@
         <v>1</v>
       </c>
       <c r="B3" t="s" s="5">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C3" t="s" s="6">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" t="s" s="6">
-        <v>161</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" ht="20.05" customHeight="1">
@@ -5056,13 +5173,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s" s="10">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="C4" t="s" s="11">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="D4" t="s" s="11">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="E4" s="13"/>
     </row>
@@ -5071,13 +5188,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="s" s="10">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C5" t="s" s="11">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="D5" t="s" s="11">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="E5" s="13"/>
     </row>
@@ -5086,13 +5203,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="s" s="10">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C6" t="s" s="11">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="D6" t="s" s="11">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="E6" s="13"/>
     </row>
@@ -5101,10 +5218,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s" s="10">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C7" t="s" s="11">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="D7" s="13"/>
       <c r="E7" s="13"/>
@@ -5114,14 +5231,14 @@
         <v>6</v>
       </c>
       <c r="B8" t="s" s="10">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" t="s" s="11">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="E8" t="s" s="28">
-        <v>129</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" ht="20.05" customHeight="1">
@@ -5129,14 +5246,14 @@
         <v>7</v>
       </c>
       <c r="B9" t="s" s="10">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="C9" s="13"/>
-      <c r="D9" t="s" s="30">
-        <v>174</v>
-      </c>
-      <c r="E9" t="s" s="31">
-        <v>132</v>
+      <c r="D9" t="s" s="31">
+        <v>181</v>
+      </c>
+      <c r="E9" t="s" s="32">
+        <v>139</v>
       </c>
     </row>
     <row r="10" ht="20.85" customHeight="1">
@@ -5144,14 +5261,14 @@
         <v>8</v>
       </c>
       <c r="B10" t="s" s="10">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="C10" s="13"/>
       <c r="D10" t="s" s="11">
-        <v>175</v>
-      </c>
-      <c r="E10" t="s" s="33">
-        <v>135</v>
+        <v>182</v>
+      </c>
+      <c r="E10" t="s" s="35">
+        <v>142</v>
       </c>
     </row>
     <row r="11" ht="21.7" customHeight="1">
@@ -5159,14 +5276,14 @@
         <v>9</v>
       </c>
       <c r="B11" t="s" s="10">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C11" s="13"/>
-      <c r="D11" t="s" s="34">
-        <v>176</v>
-      </c>
-      <c r="E11" t="s" s="35">
-        <v>138</v>
+      <c r="D11" t="s" s="36">
+        <v>183</v>
+      </c>
+      <c r="E11" t="s" s="37">
+        <v>145</v>
       </c>
     </row>
     <row r="12" ht="20.85" customHeight="1">
@@ -5174,14 +5291,14 @@
         <v>10</v>
       </c>
       <c r="B12" t="s" s="10">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" t="s" s="11">
-        <v>177</v>
-      </c>
-      <c r="E12" t="s" s="37">
-        <v>141</v>
+        <v>184</v>
+      </c>
+      <c r="E12" t="s" s="40">
+        <v>148</v>
       </c>
     </row>
     <row r="13" ht="20.05" customHeight="1">
@@ -5189,14 +5306,14 @@
         <v>11</v>
       </c>
       <c r="B13" t="s" s="10">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" t="s" s="11">
-        <v>178</v>
-      </c>
-      <c r="E13" t="s" s="39">
-        <v>144</v>
+        <v>185</v>
+      </c>
+      <c r="E13" t="s" s="43">
+        <v>151</v>
       </c>
     </row>
     <row r="14" ht="20.05" customHeight="1">
@@ -5204,14 +5321,14 @@
         <v>12</v>
       </c>
       <c r="B14" t="s" s="10">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" t="s" s="11">
-        <v>179</v>
-      </c>
-      <c r="E14" t="s" s="41">
-        <v>147</v>
+        <v>186</v>
+      </c>
+      <c r="E14" t="s" s="46">
+        <v>154</v>
       </c>
     </row>
     <row r="15" ht="20.05" customHeight="1">
@@ -5219,14 +5336,14 @@
         <v>13</v>
       </c>
       <c r="B15" t="s" s="10">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" t="s" s="11">
-        <v>180</v>
-      </c>
-      <c r="E15" t="s" s="42">
-        <v>150</v>
+        <v>187</v>
+      </c>
+      <c r="E15" t="s" s="47">
+        <v>157</v>
       </c>
     </row>
     <row r="16" ht="20.05" customHeight="1">
@@ -5234,14 +5351,14 @@
         <v>14</v>
       </c>
       <c r="B16" t="s" s="10">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="C16" s="13"/>
-      <c r="D16" t="s" s="30">
-        <v>181</v>
-      </c>
-      <c r="E16" t="s" s="44">
-        <v>153</v>
+      <c r="D16" t="s" s="31">
+        <v>188</v>
+      </c>
+      <c r="E16" t="s" s="50">
+        <v>160</v>
       </c>
     </row>
     <row r="17" ht="20.05" customHeight="1">
@@ -5249,13 +5366,13 @@
         <v>15</v>
       </c>
       <c r="B17" t="s" s="10">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="C17" t="s" s="11">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="D17" t="s" s="11">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="E17" s="13"/>
     </row>
@@ -5264,22 +5381,22 @@
         <v>16</v>
       </c>
       <c r="B18" t="s" s="10">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
     </row>
     <row r="19" ht="20.05" customHeight="1">
-      <c r="A19" s="45"/>
-      <c r="B19" s="46"/>
+      <c r="A19" s="51"/>
+      <c r="B19" s="52"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
     </row>
     <row r="20" ht="20.05" customHeight="1">
-      <c r="A20" s="45"/>
-      <c r="B20" s="46"/>
+      <c r="A20" s="51"/>
+      <c r="B20" s="52"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
       <c r="E20" s="13"/>
@@ -5304,17 +5421,17 @@
   <dimension ref="A2:E9"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="8.10156" style="48" customWidth="1"/>
-    <col min="2" max="2" width="54.8516" style="48" customWidth="1"/>
-    <col min="3" max="3" width="23.6719" style="48" customWidth="1"/>
-    <col min="4" max="4" width="26.3516" style="48" customWidth="1"/>
-    <col min="5" max="5" width="16.3516" style="48" customWidth="1"/>
-    <col min="6" max="16384" width="16.3516" style="48" customWidth="1"/>
+    <col min="1" max="1" width="8.10156" style="54" customWidth="1"/>
+    <col min="2" max="2" width="54.8516" style="54" customWidth="1"/>
+    <col min="3" max="3" width="23.6719" style="54" customWidth="1"/>
+    <col min="4" max="4" width="26.3516" style="54" customWidth="1"/>
+    <col min="5" max="5" width="16.3516" style="54" customWidth="1"/>
+    <col min="6" max="16384" width="16.3516" style="54" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.65" customHeight="1">
       <c r="A1" t="s" s="2">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5323,19 +5440,19 @@
     </row>
     <row r="2" ht="20.25" customHeight="1">
       <c r="A2" t="s" s="24">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B2" t="s" s="3">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s" s="3">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s" s="3">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E2" t="s" s="3">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" ht="20.25" customHeight="1">
@@ -5343,14 +5460,14 @@
         <v>1</v>
       </c>
       <c r="B3" t="s" s="5">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C3" t="s" s="6">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" t="s" s="6">
-        <v>187</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" ht="20.05" customHeight="1">
@@ -5358,11 +5475,11 @@
         <v>2</v>
       </c>
       <c r="B4" t="s" s="10">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" t="s" s="11">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="E4" s="13"/>
     </row>
@@ -5371,13 +5488,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="s" s="10">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="C5" t="s" s="11">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="D5" t="s" s="11">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="E5" s="13"/>
     </row>
@@ -5386,13 +5503,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="s" s="10">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="C6" t="s" s="11">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="D6" t="s" s="11">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="E6" s="13"/>
     </row>
@@ -5401,14 +5518,14 @@
         <v>5</v>
       </c>
       <c r="B7" t="s" s="10">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="C7" s="13"/>
       <c r="D7" t="s" s="11">
-        <v>196</v>
-      </c>
-      <c r="E7" t="s" s="49">
-        <v>144</v>
+        <v>203</v>
+      </c>
+      <c r="E7" t="s" s="55">
+        <v>151</v>
       </c>
     </row>
     <row r="8" ht="20.05" customHeight="1">
@@ -5416,14 +5533,14 @@
         <v>7</v>
       </c>
       <c r="B8" t="s" s="10">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" t="s" s="11">
-        <v>198</v>
-      </c>
-      <c r="E8" t="s" s="50">
-        <v>141</v>
+        <v>205</v>
+      </c>
+      <c r="E8" t="s" s="56">
+        <v>148</v>
       </c>
     </row>
     <row r="9" ht="20.05" customHeight="1">
@@ -5431,7 +5548,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s" s="10">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
@@ -5457,17 +5574,17 @@
   <dimension ref="A2:E18"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="8.10156" style="51" customWidth="1"/>
-    <col min="2" max="2" width="56.1172" style="51" customWidth="1"/>
-    <col min="3" max="3" width="23.6719" style="51" customWidth="1"/>
-    <col min="4" max="4" width="47.2422" style="51" customWidth="1"/>
-    <col min="5" max="5" width="16.3516" style="51" customWidth="1"/>
-    <col min="6" max="16384" width="16.3516" style="51" customWidth="1"/>
+    <col min="1" max="1" width="8.10156" style="57" customWidth="1"/>
+    <col min="2" max="2" width="56.1172" style="57" customWidth="1"/>
+    <col min="3" max="3" width="23.6719" style="57" customWidth="1"/>
+    <col min="4" max="4" width="47.2422" style="57" customWidth="1"/>
+    <col min="5" max="5" width="16.3516" style="57" customWidth="1"/>
+    <col min="6" max="16384" width="16.3516" style="57" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.65" customHeight="1">
       <c r="A1" t="s" s="2">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5476,19 +5593,19 @@
     </row>
     <row r="2" ht="20.25" customHeight="1">
       <c r="A2" t="s" s="24">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B2" t="s" s="3">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s" s="3">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s" s="3">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E2" t="s" s="3">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" ht="20.25" customHeight="1">
@@ -5496,14 +5613,14 @@
         <v>1</v>
       </c>
       <c r="B3" t="s" s="5">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C3" t="s" s="6">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" t="s" s="6">
-        <v>161</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" ht="20.05" customHeight="1">
@@ -5511,11 +5628,11 @@
         <v>2</v>
       </c>
       <c r="B4" t="s" s="10">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" t="s" s="11">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="E4" s="13"/>
     </row>
@@ -5524,13 +5641,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="s" s="10">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C5" t="s" s="11">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="D5" t="s" s="11">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="E5" s="13"/>
     </row>
@@ -5539,10 +5656,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s" s="10">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="C6" t="s" s="11">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
@@ -5552,11 +5669,11 @@
         <v>5</v>
       </c>
       <c r="B7" t="s" s="10">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="C7" s="13"/>
       <c r="D7" t="s" s="11">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="E7" s="13"/>
     </row>
@@ -5565,7 +5682,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s" s="10">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
@@ -5576,13 +5693,13 @@
         <v>7</v>
       </c>
       <c r="B9" t="s" s="10">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="C9" t="s" s="11">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="D9" t="s" s="11">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="E9" s="13"/>
     </row>
@@ -5591,29 +5708,29 @@
         <v>8</v>
       </c>
       <c r="B10" t="s" s="10">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="C10" t="s" s="11">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D10" t="s" s="11">
-        <v>214</v>
-      </c>
-      <c r="E10" s="52"/>
+        <v>221</v>
+      </c>
+      <c r="E10" s="58"/>
     </row>
     <row r="11" ht="20.05" customHeight="1">
       <c r="A11" s="27">
         <v>9</v>
       </c>
       <c r="B11" t="s" s="10">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" t="s" s="11">
-        <v>216</v>
-      </c>
-      <c r="E11" t="s" s="50">
-        <v>141</v>
+        <v>223</v>
+      </c>
+      <c r="E11" t="s" s="56">
+        <v>148</v>
       </c>
     </row>
     <row r="12" ht="20.05" customHeight="1">
@@ -5621,14 +5738,14 @@
         <v>10</v>
       </c>
       <c r="B12" t="s" s="10">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" t="s" s="11">
-        <v>217</v>
-      </c>
-      <c r="E12" t="s" s="39">
-        <v>144</v>
+        <v>224</v>
+      </c>
+      <c r="E12" t="s" s="43">
+        <v>151</v>
       </c>
     </row>
     <row r="13" ht="20.05" customHeight="1">
@@ -5636,14 +5753,14 @@
         <v>11</v>
       </c>
       <c r="B13" t="s" s="10">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" t="s" s="11">
-        <v>218</v>
-      </c>
-      <c r="E13" t="s" s="41">
-        <v>147</v>
+        <v>225</v>
+      </c>
+      <c r="E13" t="s" s="46">
+        <v>154</v>
       </c>
     </row>
     <row r="14" ht="20.05" customHeight="1">
@@ -5651,14 +5768,14 @@
         <v>12</v>
       </c>
       <c r="B14" t="s" s="10">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" t="s" s="11">
-        <v>219</v>
-      </c>
-      <c r="E14" t="s" s="42">
-        <v>150</v>
+        <v>226</v>
+      </c>
+      <c r="E14" t="s" s="47">
+        <v>157</v>
       </c>
     </row>
     <row r="15" ht="20.05" customHeight="1">
@@ -5666,14 +5783,14 @@
         <v>13</v>
       </c>
       <c r="B15" t="s" s="10">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="C15" s="13"/>
-      <c r="D15" t="s" s="30">
-        <v>220</v>
-      </c>
-      <c r="E15" t="s" s="44">
-        <v>153</v>
+      <c r="D15" t="s" s="31">
+        <v>227</v>
+      </c>
+      <c r="E15" t="s" s="50">
+        <v>160</v>
       </c>
     </row>
     <row r="16" ht="20.05" customHeight="1">
@@ -5681,22 +5798,22 @@
         <v>14</v>
       </c>
       <c r="B16" t="s" s="10">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
       <c r="E16" s="13"/>
     </row>
     <row r="17" ht="20.05" customHeight="1">
-      <c r="A17" s="45"/>
-      <c r="B17" s="46"/>
+      <c r="A17" s="51"/>
+      <c r="B17" s="52"/>
       <c r="C17" s="13"/>
       <c r="D17" s="13"/>
       <c r="E17" s="13"/>
     </row>
     <row r="18" ht="20.05" customHeight="1">
-      <c r="A18" s="45"/>
-      <c r="B18" s="46"/>
+      <c r="A18" s="51"/>
+      <c r="B18" s="52"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
@@ -5721,10 +5838,10 @@
   <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="16.3516" style="53" customWidth="1"/>
-    <col min="2" max="2" width="35.1484" style="53" customWidth="1"/>
-    <col min="3" max="5" width="16.3516" style="53" customWidth="1"/>
-    <col min="6" max="16384" width="16.3516" style="53" customWidth="1"/>
+    <col min="1" max="1" width="16.3516" style="59" customWidth="1"/>
+    <col min="2" max="2" width="35.1484" style="59" customWidth="1"/>
+    <col min="3" max="5" width="16.3516" style="59" customWidth="1"/>
+    <col min="6" max="16384" width="16.3516" style="59" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20.25" customHeight="1">
@@ -5735,70 +5852,70 @@
       <c r="E1" s="25"/>
     </row>
     <row r="2" ht="20.25" customHeight="1">
-      <c r="A2" s="54"/>
+      <c r="A2" s="60"/>
       <c r="B2" t="s" s="5">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C2" s="8"/>
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
     <row r="3" ht="32.05" customHeight="1">
-      <c r="A3" s="55"/>
+      <c r="A3" s="61"/>
       <c r="B3" t="s" s="10">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
       <c r="E3" s="13"/>
     </row>
     <row r="4" ht="32.05" customHeight="1">
-      <c r="A4" s="55"/>
+      <c r="A4" s="61"/>
       <c r="B4" t="s" s="10">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
     </row>
     <row r="5" ht="20.05" customHeight="1">
-      <c r="A5" s="55"/>
-      <c r="B5" s="46"/>
+      <c r="A5" s="61"/>
+      <c r="B5" s="52"/>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
     </row>
     <row r="6" ht="20.05" customHeight="1">
-      <c r="A6" s="55"/>
-      <c r="B6" s="46"/>
+      <c r="A6" s="61"/>
+      <c r="B6" s="52"/>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
     </row>
     <row r="7" ht="20.05" customHeight="1">
-      <c r="A7" s="55"/>
-      <c r="B7" s="46"/>
+      <c r="A7" s="61"/>
+      <c r="B7" s="52"/>
       <c r="C7" s="13"/>
       <c r="D7" s="13"/>
       <c r="E7" s="13"/>
     </row>
     <row r="8" ht="20.05" customHeight="1">
-      <c r="A8" s="55"/>
-      <c r="B8" s="46"/>
+      <c r="A8" s="61"/>
+      <c r="B8" s="52"/>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
     </row>
     <row r="9" ht="20.05" customHeight="1">
-      <c r="A9" s="55"/>
-      <c r="B9" s="46"/>
+      <c r="A9" s="61"/>
+      <c r="B9" s="52"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
     </row>
     <row r="10" ht="20.05" customHeight="1">
-      <c r="A10" s="55"/>
-      <c r="B10" s="46"/>
+      <c r="A10" s="61"/>
+      <c r="B10" s="52"/>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
@@ -5820,17 +5937,17 @@
   <dimension ref="A2:E20"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="8.10156" style="56" customWidth="1"/>
-    <col min="2" max="2" width="57.1719" style="56" customWidth="1"/>
-    <col min="3" max="3" width="33.8125" style="56" customWidth="1"/>
-    <col min="4" max="4" width="35.0781" style="56" customWidth="1"/>
-    <col min="5" max="5" width="16.3516" style="56" customWidth="1"/>
-    <col min="6" max="16384" width="16.3516" style="56" customWidth="1"/>
+    <col min="1" max="1" width="8.10156" style="62" customWidth="1"/>
+    <col min="2" max="2" width="57.1719" style="62" customWidth="1"/>
+    <col min="3" max="3" width="33.8125" style="62" customWidth="1"/>
+    <col min="4" max="4" width="35.0781" style="62" customWidth="1"/>
+    <col min="5" max="5" width="16.3516" style="62" customWidth="1"/>
+    <col min="6" max="16384" width="16.3516" style="62" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.65" customHeight="1">
       <c r="A1" t="s" s="2">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5839,19 +5956,19 @@
     </row>
     <row r="2" ht="20.25" customHeight="1">
       <c r="A2" t="s" s="24">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B2" t="s" s="3">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s" s="3">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s" s="3">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E2" t="s" s="3">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" ht="20.25" customHeight="1">
@@ -5859,14 +5976,14 @@
         <v>1</v>
       </c>
       <c r="B3" t="s" s="5">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C3" t="s" s="6">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" t="s" s="6">
-        <v>161</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" ht="20.05" customHeight="1">
@@ -5874,11 +5991,11 @@
         <v>2</v>
       </c>
       <c r="B4" t="s" s="10">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" t="s" s="11">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="E4" s="13"/>
     </row>
@@ -5887,7 +6004,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s" s="10">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
@@ -5898,11 +6015,11 @@
         <v>4</v>
       </c>
       <c r="B6" t="s" s="10">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" t="s" s="11">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="E6" s="13"/>
     </row>
@@ -5911,13 +6028,13 @@
         <v>5</v>
       </c>
       <c r="B7" t="s" s="10">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="C7" t="s" s="11">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="D7" t="s" s="11">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="E7" s="13"/>
     </row>
@@ -5926,16 +6043,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s" s="10">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C8" t="s" s="11">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D8" t="s" s="11">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="E8" t="s" s="28">
-        <v>129</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" ht="20.05" customHeight="1">
@@ -5943,16 +6060,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s" s="10">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="C9" t="s" s="11">
-        <v>230</v>
-      </c>
-      <c r="D9" t="s" s="30">
-        <v>232</v>
-      </c>
-      <c r="E9" t="s" s="31">
-        <v>132</v>
+        <v>237</v>
+      </c>
+      <c r="D9" t="s" s="31">
+        <v>239</v>
+      </c>
+      <c r="E9" t="s" s="32">
+        <v>139</v>
       </c>
     </row>
     <row r="10" ht="20.85" customHeight="1">
@@ -5960,16 +6077,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="s" s="10">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="C10" t="s" s="11">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D10" t="s" s="11">
-        <v>233</v>
-      </c>
-      <c r="E10" t="s" s="33">
-        <v>135</v>
+        <v>240</v>
+      </c>
+      <c r="E10" t="s" s="35">
+        <v>142</v>
       </c>
     </row>
     <row r="11" ht="21.7" customHeight="1">
@@ -5977,16 +6094,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s" s="10">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C11" t="s" s="11">
-        <v>230</v>
-      </c>
-      <c r="D11" t="s" s="34">
-        <v>234</v>
-      </c>
-      <c r="E11" t="s" s="35">
-        <v>138</v>
+        <v>237</v>
+      </c>
+      <c r="D11" t="s" s="36">
+        <v>241</v>
+      </c>
+      <c r="E11" t="s" s="37">
+        <v>145</v>
       </c>
     </row>
     <row r="12" ht="20.85" customHeight="1">
@@ -5994,16 +6111,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s" s="10">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="C12" t="s" s="11">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D12" t="s" s="11">
-        <v>235</v>
-      </c>
-      <c r="E12" t="s" s="37">
-        <v>141</v>
+        <v>242</v>
+      </c>
+      <c r="E12" t="s" s="40">
+        <v>148</v>
       </c>
     </row>
     <row r="13" ht="20.05" customHeight="1">
@@ -6011,16 +6128,16 @@
         <v>11</v>
       </c>
       <c r="B13" t="s" s="10">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C13" t="s" s="11">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D13" t="s" s="11">
-        <v>236</v>
-      </c>
-      <c r="E13" t="s" s="39">
-        <v>144</v>
+        <v>243</v>
+      </c>
+      <c r="E13" t="s" s="43">
+        <v>151</v>
       </c>
     </row>
     <row r="14" ht="20.05" customHeight="1">
@@ -6028,16 +6145,16 @@
         <v>12</v>
       </c>
       <c r="B14" t="s" s="10">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="C14" t="s" s="11">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D14" t="s" s="11">
-        <v>237</v>
-      </c>
-      <c r="E14" t="s" s="41">
-        <v>147</v>
+        <v>244</v>
+      </c>
+      <c r="E14" t="s" s="46">
+        <v>154</v>
       </c>
     </row>
     <row r="15" ht="20.05" customHeight="1">
@@ -6045,16 +6162,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="s" s="10">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C15" t="s" s="11">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D15" t="s" s="11">
-        <v>238</v>
-      </c>
-      <c r="E15" t="s" s="57">
-        <v>150</v>
+        <v>245</v>
+      </c>
+      <c r="E15" t="s" s="63">
+        <v>157</v>
       </c>
     </row>
     <row r="16" ht="20.05" customHeight="1">
@@ -6062,7 +6179,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="s" s="10">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
@@ -6073,11 +6190,11 @@
         <v>15</v>
       </c>
       <c r="B17" t="s" s="10">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="C17" s="13"/>
       <c r="D17" t="s" s="11">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="E17" s="13"/>
     </row>
@@ -6086,22 +6203,22 @@
         <v>16</v>
       </c>
       <c r="B18" t="s" s="10">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
     </row>
     <row r="19" ht="20.05" customHeight="1">
-      <c r="A19" s="45"/>
-      <c r="B19" s="46"/>
+      <c r="A19" s="51"/>
+      <c r="B19" s="52"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
     </row>
     <row r="20" ht="20.05" customHeight="1">
-      <c r="A20" s="45"/>
-      <c r="B20" s="46"/>
+      <c r="A20" s="51"/>
+      <c r="B20" s="52"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
       <c r="E20" s="13"/>
@@ -6126,17 +6243,17 @@
   <dimension ref="A2:E15"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="8.10156" style="58" customWidth="1"/>
-    <col min="2" max="2" width="32.6719" style="58" customWidth="1"/>
-    <col min="3" max="3" width="23.6719" style="58" customWidth="1"/>
-    <col min="4" max="4" width="24.625" style="58" customWidth="1"/>
-    <col min="5" max="5" width="16.3516" style="58" customWidth="1"/>
-    <col min="6" max="16384" width="16.3516" style="58" customWidth="1"/>
+    <col min="1" max="1" width="8.10156" style="64" customWidth="1"/>
+    <col min="2" max="2" width="32.6719" style="64" customWidth="1"/>
+    <col min="3" max="3" width="23.6719" style="64" customWidth="1"/>
+    <col min="4" max="4" width="24.625" style="64" customWidth="1"/>
+    <col min="5" max="5" width="16.3516" style="64" customWidth="1"/>
+    <col min="6" max="16384" width="16.3516" style="64" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.65" customHeight="1">
       <c r="A1" t="s" s="2">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6145,19 +6262,19 @@
     </row>
     <row r="2" ht="20.25" customHeight="1">
       <c r="A2" t="s" s="24">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B2" t="s" s="3">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s" s="3">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s" s="3">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E2" t="s" s="3">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" ht="20.25" customHeight="1">
@@ -6165,14 +6282,14 @@
         <v>1</v>
       </c>
       <c r="B3" t="s" s="5">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C3" t="s" s="6">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" t="s" s="6">
-        <v>187</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" ht="20.05" customHeight="1">
@@ -6180,11 +6297,11 @@
         <v>2</v>
       </c>
       <c r="B4" t="s" s="10">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" t="s" s="11">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="E4" s="13"/>
     </row>
@@ -6193,13 +6310,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="s" s="10">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C5" t="s" s="11">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="D5" t="s" s="11">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="E5" s="13"/>
     </row>
@@ -6208,7 +6325,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s" s="10">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
@@ -6219,11 +6336,11 @@
         <v>5</v>
       </c>
       <c r="B7" t="s" s="10">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="C7" s="13"/>
       <c r="D7" t="s" s="11">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="E7" s="13"/>
     </row>
@@ -6232,11 +6349,11 @@
         <v>6</v>
       </c>
       <c r="B8" t="s" s="10">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" t="s" s="11">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="E8" s="13"/>
     </row>
@@ -6245,11 +6362,11 @@
         <v>7</v>
       </c>
       <c r="B9" t="s" s="10">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="C9" s="13"/>
       <c r="D9" t="s" s="11">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="E9" s="13"/>
     </row>
@@ -6258,14 +6375,14 @@
         <v>8</v>
       </c>
       <c r="B10" t="s" s="10">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C10" s="13"/>
       <c r="D10" t="s" s="11">
-        <v>255</v>
-      </c>
-      <c r="E10" t="s" s="39">
-        <v>144</v>
+        <v>262</v>
+      </c>
+      <c r="E10" t="s" s="43">
+        <v>151</v>
       </c>
     </row>
     <row r="11" ht="20.05" customHeight="1">
@@ -6273,16 +6390,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s" s="10">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="C11" t="s" s="11">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="D11" t="s" s="11">
-        <v>257</v>
-      </c>
-      <c r="E11" t="s" s="41">
-        <v>147</v>
+        <v>264</v>
+      </c>
+      <c r="E11" t="s" s="46">
+        <v>154</v>
       </c>
     </row>
     <row r="12" ht="20.05" customHeight="1">
@@ -6290,16 +6407,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s" s="10">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="C12" t="s" s="11">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="D12" t="s" s="11">
-        <v>259</v>
-      </c>
-      <c r="E12" t="s" s="57">
-        <v>150</v>
+        <v>266</v>
+      </c>
+      <c r="E12" t="s" s="63">
+        <v>157</v>
       </c>
     </row>
     <row r="13" ht="20.05" customHeight="1">
@@ -6307,22 +6424,22 @@
         <v>11</v>
       </c>
       <c r="B13" t="s" s="10">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
     </row>
     <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" s="45"/>
-      <c r="B14" s="46"/>
+      <c r="A14" s="51"/>
+      <c r="B14" s="52"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
     </row>
     <row r="15" ht="20.05" customHeight="1">
-      <c r="A15" s="45"/>
-      <c r="B15" s="46"/>
+      <c r="A15" s="51"/>
+      <c r="B15" s="52"/>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
       <c r="E15" s="13"/>

</xml_diff>